<commit_message>
Sync the HeritageGraph-LUX migration folder to the current ontology
Same layout and method as the imported repository; only what the current
HeritageGraph requires is changed: namespace, ontology download path, every
HeritageGraph term resolved to its v1.0.0 IRI (renamed and removed terms
included), the alignment adapted (LUX-facing targets follow the Linked Art
context), migration/validation SPARQL and migrator templates, and the mapping
workbook regenerated with mapping/build_mapping.py. Historical run reports
are left unchanged.
</commit_message>
<xml_diff>
--- a/heritagegraph-lux-migration/mapping/HeritageGraph_LUX_Mapping.xlsx
+++ b/heritagegraph-lux-migration/mapping/HeritageGraph_LUX_Mapping.xlsx
@@ -845,7 +845,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>equivalentClass</t>
+          <t>subClassOf</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr"/>
@@ -905,7 +905,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>equivalentClass</t>
+          <t>dropped in v1.0.0</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>BuddhistMonument</t>
+          <t>ReligiousStructure</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>BuddhistMonument</t>
+          <t>ReligiousStructure</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1129,12 +1129,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>subClassOf</t>
+          <t>removed in v1.0.0</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Modeled with type assignment in LUX.</t>
+          <t>Modeled with type assignment in LUX. Class not in HeritageGraph v1.0.0.</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1729,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>LivingGoddessSelection</t>
+          <t>KumariSelectionEvent</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
@@ -1754,14 +1754,14 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Novel HG event.</t>
+          <t>Novel HG event. Renamed from LivingGoddessSelection in v1.0.0.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>LivingGoddessRetirement</t>
+          <t>KumariRetirementEvent</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -1786,14 +1786,14 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>Novel HG event.</t>
+          <t>Novel HG event. Renamed from LivingGoddessRetirement in v1.0.0.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>LivingGoddessTenure</t>
+          <t>KumariTenure</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -1816,7 +1816,11 @@
           <t>subClassOf</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Renamed from LivingGoddessTenure in v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -2093,7 +2097,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>HeritageAssertion</t>
+          <t>Assertion</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -2113,12 +2117,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>subClassOf</t>
+          <t>none (v1.0.0 uses crminf:I2_Belief)</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>LUX uses E13 inside provenance/identification.</t>
+          <t>LUX uses E13 inside provenance/identification. Renamed from HeritageAssertion in v1.0.0.</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2161,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>AssertableEntity</t>
+          <t>AssertionSubject</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -2182,7 +2186,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Abstract; LUX has no equivalent. Keep CRMinf alignment.</t>
+          <t>Abstract; LUX has no equivalent. Keep CRMinf alignment. Renamed from AssertableEntity in v1.0.0.</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2230,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>PropositionalObject</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -2273,7 +2277,7 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>broadMatch</t>
+          <t>dropped in v1.0.0</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
@@ -2381,7 +2385,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>DatePrecisionEnum</t>
+          <t>DatePrecision</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -2406,14 +2410,14 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Enum -&gt; SKOS ConceptScheme of Type instances.</t>
+          <t>Enum -&gt; SKOS ConceptScheme of Type instances. Renamed from DatePrecisionEnum in v1.0.0.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>ConditionTypeEnum</t>
+          <t>ConditionType</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -2436,12 +2440,16 @@
           <t>subClassOf</t>
         </is>
       </c>
-      <c r="F62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Renamed from ConditionTypeEnum in v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>ExistenceStatusEnum</t>
+          <t>ExistenceStatus</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -2464,12 +2472,16 @@
           <t>subClassOf</t>
         </is>
       </c>
-      <c r="F63" s="3" t="inlineStr"/>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Renamed from ExistenceStatusEnum in v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>GuthiTypeEnum</t>
+          <t>GuthiType</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -2492,12 +2504,16 @@
           <t>subClassOf</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Renamed from GuthiTypeEnum in v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>RitualTypeEnum</t>
+          <t>RitualType</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -2520,12 +2536,16 @@
           <t>subClassOf</t>
         </is>
       </c>
-      <c r="F65" s="3" t="inlineStr"/>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Renamed from RitualTypeEnum in v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>SyncreticTypeEnum</t>
+          <t>SyncreticType</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -2548,7 +2568,11 @@
           <t>subClassOf</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Renamed from SyncreticTypeEnum in v1.0.0.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2659,7 +2683,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
@@ -2687,7 +2711,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -2775,7 +2799,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>closeMatch</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
@@ -2863,7 +2887,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr"/>
@@ -2891,7 +2915,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr"/>
@@ -2919,7 +2943,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
@@ -2979,7 +3003,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -3011,7 +3035,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr"/>
@@ -3039,7 +3063,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>none (v1.0.0 uses crm:P53i_is_former_or_current_location_of)</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr"/>
@@ -3067,7 +3091,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>none (v1.0.0 uses crm:P125_used_object_of_type)</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr"/>
@@ -3095,7 +3119,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>none (v1.0.0 uses crm:P33_used_specific_technique)</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr"/>
@@ -3108,7 +3132,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>crm:E55_Type</t>
+          <t>ArchitecturalStyle</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -3136,7 +3160,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ConditionTypeEnum</t>
+          <t>ConditionType</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3192,7 +3216,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>GuthiTypeEnum</t>
+          <t>GuthiType</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3220,7 +3244,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>RitualTypeEnum</t>
+          <t>RitualType</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -3263,7 +3287,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>seeAlso</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -3295,7 +3319,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>seeAlso</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr"/>
@@ -3308,7 +3332,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>SyncreticTypeEnum</t>
+          <t>SyncreticType</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -3336,7 +3360,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>DatePrecisionEnum</t>
+          <t>DatePrecision</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -3379,10 +3403,14 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3392,7 +3420,7 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>ExistenceStatusEnum</t>
+          <t>ExistenceStatus</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -3435,7 +3463,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
@@ -3463,7 +3491,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr"/>
@@ -3519,7 +3547,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr"/>
@@ -3547,7 +3575,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr"/>
@@ -3603,7 +3631,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr"/>
@@ -3631,7 +3659,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>none (v1.0.0 uses crm:P50i_is_current_keeper_of)</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr"/>
@@ -3659,7 +3687,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr"/>
@@ -3687,7 +3715,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr"/>
@@ -3867,7 +3895,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>produced_information_object</t>
+          <t>generated</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -3887,15 +3915,19 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
+          <t>none (v1.0.0 uses prov:generated)</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Renamed from produced_information_object in v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>created_by_documentation</t>
+          <t>was_generated_by</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -3915,10 +3947,14 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="inlineStr"/>
+          <t>none (v1.0.0 uses prov:wasGeneratedBy)</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Renamed from created_by_documentation in v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3943,10 +3979,14 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
@@ -3971,10 +4011,14 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
-        </is>
-      </c>
-      <c r="F49" s="3" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3999,10 +4043,14 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
@@ -4027,10 +4075,14 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F51" s="3" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4055,7 +4107,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr"/>
@@ -4083,7 +4135,7 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr"/>
@@ -4111,10 +4163,14 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
@@ -4139,7 +4195,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F55" s="3" t="inlineStr"/>
@@ -4167,7 +4223,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>none (v1.0.0 uses crm:P62_depicts)</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -4227,7 +4283,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>none (v1.0.0 uses crm:P62i_is_depicted_by)</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr"/>
@@ -4255,7 +4311,7 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>none (v1.0.0 uses rdfs:label)</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -4287,7 +4343,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>none (v1.0.0 uses dcterms:identifier)</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr"/>
@@ -4315,7 +4371,7 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>identity (direct URI reuse)</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr"/>
@@ -4343,7 +4399,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>seeAlso</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr"/>
@@ -4403,7 +4459,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>none (v1.0.0 uses geo:asWKT)</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr"/>
@@ -4431,15 +4487,19 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F65" s="3" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>was_attributed_to_agent</t>
+          <t>was_attributed_to</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -4459,10 +4519,14 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr"/>
+          <t>none (v1.0.0 uses prov:wasAttributedTo)</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Renamed from was_attributed_to_agent in v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
@@ -4487,10 +4551,14 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F67" s="3" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4515,10 +4583,14 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr"/>
+          <t>removed in v1.0.0</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Property not in HeritageGraph v1.0.0.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
@@ -4556,7 +4628,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>xsd:float</t>
+          <t>xsd:decimal</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -4860,7 +4932,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Generic period (Lichhavi, Malla, Shah, Rana). LivingGoddessTenure becomes its subclass.</t>
+          <t>Generic period (Lichhavi, Malla, Shah, Rana). KumariTenure becomes its subclass.</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6544,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Generic historical period. hg:LivingGoddessTenure becomes its subclass.</t>
+          <t>Generic historical period. hg:KumariTenure becomes its subclass.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Repair conservativity violations in the LUX module and add a lux-conservativity gate
- evaluation/reasoning_extras.py lux-conservativity (make check, CI): probe instances
  of every class/property pair the module maps, classified with the module and
  CIDOC-CRM 7.1.3 (+ CRMinf, CRMsci), must respect CRM's disjointness (E2/E77 stated in
  the E2 scope note; E18/E28 from the scope notes) and gain no core class that core +
  CIDOC-CRM alone do not entail. Negative control: re-adding
  documentedBy ⊑ crm:P94i_was_created_by is caught (30 violations).
- Module repairs: documentedBy, managedByGuthi, isAboutDeity, birthTimespan,
  deathTimespan, publicationTimespan, hasDataCustodian → skos:closeMatch;
  mentionedInSource ≡ crm:P67i → rdfs:subPropertyOf; hg:Activity ⊑ hg:HistoricalEvent
  and Metadata ⊑ hg:InformationObject removed.
- Regenerated the mapping workbook, LUX report and alignment graph.
</commit_message>
<xml_diff>
--- a/heritagegraph-lux-migration/mapping/HeritageGraph_LUX_Mapping.xlsx
+++ b/heritagegraph-lux-migration/mapping/HeritageGraph_LUX_Mapping.xlsx
@@ -3743,7 +3743,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>closeMatch</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr"/>
@@ -3771,7 +3771,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>closeMatch</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -3803,7 +3803,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>closeMatch</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr"/>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>closeMatch</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr"/>
@@ -3859,7 +3859,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>equivalentProperty</t>
+          <t>subPropertyOf</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr"/>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>closeMatch</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr"/>
@@ -4255,7 +4255,7 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>subPropertyOf</t>
+          <t>closeMatch</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr"/>

</xml_diff>